<commit_message>
Add Model Harnesses & Tools tab: per-model harness and tool matrix
- New workbook sheet covering 20 models: first-party harness/agent surface,
  third-party harness compatibility, built-in tool suites, input modalities,
  and API feature flags (function calling, parallel tool calls, structured
  outputs, reasoning controls) joined from the OpenRouter catalog snapshot
- Notes Kimi K3 weights shipped on Hugging Face 2026-07-27 as promised
- CSV export data/csv/model_harnesses_tools.csv (also included in the
  llm_data_tables.xlsx compilation); README documentation

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/llm_data_tables.xlsx
+++ b/data/llm_data_tables.xlsx
@@ -11,22 +11,24 @@
     <sheet name="cloud_provider_split" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="harness_rl_environments" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="model_comparison" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="open_vs_closed_summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="params_benchmarks" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="quantization_kld" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="tool_use_benchmarks" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="training_data" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="model_harnesses_tools" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="open_vs_closed_summary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="params_benchmarks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="quantization_kld" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="tool_use_benchmarks" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="training_data" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'by_developer'!$A$1:$F$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'cloud_provider_split'!$A$1:$I$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'harness_rl_environments'!$A$1:$J$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'model_comparison'!$A$1:$P$305</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'open_vs_closed_summary'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'params_benchmarks'!$A$1:$S$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'quantization_kld'!$A$1:$J$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'tool_use_benchmarks'!$A$1:$M$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'training_data'!$A$1:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'model_harnesses_tools'!$A$1:$N$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'open_vs_closed_summary'!$A$1:$J$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'params_benchmarks'!$A$1:$S$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'quantization_kld'!$A$1:$J$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'tool_use_benchmarks'!$A$1:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'training_data'!$A$1:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1659,6 +1661,631 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>developer</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>total_params_b</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>pretraining_tokens_t</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>tokens_per_total_param</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>disclosure_status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Undisclosed (tech report due with weights, 2026-07-27)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Pipeline disclosed without quantities: web+code+vision pretraining, long-context mid-training toward 1M, SFT, RLVR. Predecessor Kimi K2 (1T params) disclosed 15.5T tokens, so K3's corpus is presumably well beyond that; treat any specific figure circulating now as an estimate.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>kimi.com/blog/kimi-k3; Kimi K2 paper (arXiv:2507.20534)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Kimi K2 / K2.6</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Disclosed for K2 base (K2.6/K2.7 increments not broken out)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>15.5T curated tokens across web text, code, mathematics, knowledge; MuonClip optimizer, 4,096-token pretraining window.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Kimi K2 paper (arXiv:2507.20534)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Claude Fable 5</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Anthropic discloses neither corpus size nor parameter count for any frontier model.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Fable 5 system card (no training-data quantities)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Sol</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>OpenAI stopped disclosing training-data scale after GPT-3 (300B tokens, 2020). gpt-oss open-weight models also ship without a precise token count ('trillions of tokens').</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>GPT-5.6 launch materials (no training-data quantities)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Gemini 3.x</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>No corpus quantities disclosed for the Gemini series.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Gemini model cards</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GLM-5 / 5.1 / 5.2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Z.ai (Zhipu)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>753</v>
+      </c>
+      <c r="E7" t="n">
+        <v>27</v>
+      </c>
+      <c r="F7" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Disclosed (GLM-5 base, which 5.1/5.2 build on)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>27T-token corpus prioritizing code and reasoning early; distinct mid-training phase extends context 4K-&gt;200K with long-context agentic data.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>GLM-5 paper (arXiv:2602.15763)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Pro</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E8" t="n">
+        <v>32</v>
+      </c>
+      <c r="F8" t="n">
+        <v>20</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Disclosed ('more than 32T tokens', shared corpus with Flash)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Agentic tool-use data injected already in mid-training; FP8-mixed pretraining with MXFP4 on expert weights.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4 report (arXiv:2606.19348)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>284</v>
+      </c>
+      <c r="E9" t="n">
+        <v>32</v>
+      </c>
+      <c r="F9" t="n">
+        <v>112.7</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Disclosed ('more than 32T tokens', shared corpus with Pro)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Same &gt;32T corpus as V4 Pro; the small variant is heavily over-trained relative to its size (~113 tokens per param).</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4 report (arXiv:2606.19348)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Qwen3.7 Max</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Alibaba (Qwen)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Undisclosed (closed tier)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Alibaba disclosed 36T tokens for the open Qwen3 generation (2025) but publishes no quantities for the closed Max tier.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Qwen3 technical report (2025); Qwen3.7 launch blog</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Nemotron 3 (Nano/Super/Ultra)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>25</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Disclosed AND largely released - the only lab that ships much of the corpus itself</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>25T tokens in two phases (23.5T diverse + 1.5T high-quality) + 121B long-context phase; 16 data categories. ~8-10T tokens (~40-50% of the blend) released as open datasets (Nemotron-CC-v2.x, CC-Math, Pretraining-Code, Specialized). Documented for Nano/Super; Ultra follows the same data program.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NVIDIA Nemotron 3 pretraining docs + Nano tech report; HF Nemotron pretraining dataset collections</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MiMo-V2.5</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Xiaomi</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>310</v>
+      </c>
+      <c r="E12" t="n">
+        <v>48</v>
+      </c>
+      <c r="F12" t="n">
+        <v>154.8</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Disclosed - largest disclosed corpus of any model here</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>~48T tokens, FP8 mixed precision, five-stage pipeline (text pretraining, projector warmup, multimodal pretraining, SFT/agentic post-training with 32K-&gt;256K-&gt;1M context extension, RL+MOPD). ~155 tokens per param - the most over-trained large model on this list.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>XiaomiMiMo/MiMo-V2.5 HF card; mimo.xiaomi.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hy3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tencent</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>295</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>295B/21B MoE (192 experts, top-8 routing); Tencent's model card discusses post-training scale-up but no corpus count.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Tencent Hy3 model card; SiliconFlow explainer</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MiniMax M3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>No corpus size published for M3; total params also not officially stated (third-party estimates ~200-400B).</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>M3 launch materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Llama 4 Scout</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>109</v>
+      </c>
+      <c r="E15" t="n">
+        <v>40</v>
+      </c>
+      <c r="F15" t="n">
+        <v>367</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Disclosed (2025)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>~40T multimodal tokens - highest tokens-per-param ratio here (~367x); 10M-token context via iRoPE.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Meta Llama 4 launch blog (2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Llama 4 Maverick</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>400</v>
+      </c>
+      <c r="E16" t="n">
+        <v>22</v>
+      </c>
+      <c r="F16" t="n">
+        <v>55</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Disclosed (2025)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>~22T multimodal tokens.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Meta Llama 4 launch blog (2025)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I16"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -21910,6 +22537,1469 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>developer</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>first_party_harness</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>third_party_harness_compatibility</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>builtin_tools</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>input_modalities</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>function_calling</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>parallel_tool_calls</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>structured_outputs</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>reasoning_controls</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>context_tokens</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>weekly_tokens</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MoonshotAI: Kimi K3</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Kimi Code CLI; Kimi.com / Kimi Work apps; K3 Swarm Max orchestrator (up to 300 parallel sub-agents)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Claude Code, Cursor, OpenClaw via Anthropic/OpenAI-compatible API - but requires preserved thinking history (verified harnesses only; no mid-session model switches)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Web search/fetch, terminal, code execution, vision-in-the-loop (live screenshots), video editing, Widgets + Dashboard in Kimi Work; MCP</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>image+text</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>1048576</v>
+      </c>
+      <c r="M2" t="n">
+        <v>12051888516</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Weights live on HF since 2026-07-27 (96 shards, ~99K downloads in 2 days); day-0 vLLM support with Moonshot-contributed KDA prefix caching.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MoonshotAI: Kimi K2.6</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Kimi CLI; native Agent Swarm (300 sub-agents, 4,000 steps)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Claude Code, OpenClaw, Cline (Anthropic/OpenAI-compatible)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Web search, terminal, code execution, swarm orchestration; MCP; one of only two models here exposing parallel tool calls on OpenRouter</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>image+text</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>262144</v>
+      </c>
+      <c r="M3" t="n">
+        <v>295806133970</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Apache-2.0-style open weights available now; HLE-with-tools 54.0 led all frontier models at release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Anthropic: Claude Fable 5</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Claude Code (CLI + SDK) - the industry reference harness; Claude Cowork for knowledge work</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Anthropic API only; broad ecosystem targets it (Cursor, OpenClaw, Cline all speak Anthropic protocol)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Memory tool, code execution, computer use, web search, programmatic tool calling, context editing / tool-result clearing, compaction, task budgets (beta); MCP. Adaptive thinking always on (effort parameter); no assistant prefill</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>file+image+text</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M4" t="n">
+        <v>375285408732</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Safety classifiers can reroute cyber/bio/distillation requests to Opus 4.8 (fallback affects &lt;5% of sessions per Anthropic).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Anthropic: Claude Sonnet 5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Claude Code; Claude.ai apps</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Anthropic API ecosystem (same as Fable 5)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Same Claude tool suite: memory tool, code execution, computer use, web search, compaction; MCP</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>file+image+text</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M5" t="n">
+        <v>936723011167</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Mid-tier workhorse at intro pricing ($2/$10 through Aug 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>OpenAI: GPT-5.6 Sol</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Codex suite: CLI, Cloud, VS Code extension, App Server (JSON-RPC); ChatGPT agent surfaces</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Responses API; community proxies run it inside Claude Code (some report it codes better there - model/harness entanglement debate)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Web search, code interpreter, file search, computer use (OSWorld 2.0 SOTA 62.6%), subagent orchestration (Sol as orchestrator over Terra/Luna; config bug openai/codex#31814), automatic compaction; MCP</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>file+image+text</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="M6" t="n">
+        <v>411249519808</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Models explicitly tuned for the Codex harness; ~25h uninterrupted runs reported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OpenAI: GPT-5.5</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Codex suite (previous flagship)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Responses API ecosystem</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Web search, code interpreter, file search, computer use; MCP</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>file+image+text</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="M7" t="n">
+        <v>677882959419</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Superseded by GPT-5.6 family for agentic work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Z.ai: GLM 5.2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Z.ai (Zhipu)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>None of its own - by design. GLM Coding Plan ($3-80/mo) plugs into third-party harnesses</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Claude Code (Anthropic-native API), OpenClaw, Cline, Cursor; drop-in config documented by Z.ai</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Function calling with parallel tool calls; dynamic working-memory management for thousands-of-tool-call sessions; MCP</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1048576</v>
+      </c>
+      <c r="M8" t="n">
+        <v>3515340760024</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Strongest open-weights MCP Atlas score (82.6 on Moonshot's table; 77.0 per Z.ai's own blog).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DeepSeek: DeepSeek V4 Pro</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>None - dual-mode OpenAI + Anthropic-compatible API</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Codex-style and Claude Code-style harnesses both work; popular in Kilo Code, OpenClaw, aggregators</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Function calling via new XML-based DSML schema (replaces JSON); three reasoning modes (non-think/high/max); MCP</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>1048576</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2473441480536</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Agentic tool-use data injected in mid-training, not just post-training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DeepSeek: DeepSeek V4 Flash</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>None - same dual-mode API as V4 Pro</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Same as V4 Pro; the default budget model in many third-party coding agents</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Same DSML function calling and reasoning modes; MCP</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>1048576</v>
+      </c>
+      <c r="M10" t="n">
+        <v>5240398974088</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Highest real-world tool-call volume of any paid model on OpenRouter (~70M calls/week).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MiniMax: MiniMax M3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MiniMax Agent product; no dedicated CLI</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>OpenAI/Anthropic-compatible API</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Native computer use (only open model here with it), video input in tool workflows, function calling; MCP; 24h autonomous runs with ~2,000 tool calls reported</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>image+text+video</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>1048576</v>
+      </c>
+      <c r="M11" t="n">
+        <v>3951536497593</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Multimodal agent focus (text+image+video input).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NVIDIA: Nemotron 3 Ultra</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NVIDIA API / NIM; NeMo Gym ships out-of-the-box harnesses (incl. Claude Code and Hermes) for eval/training</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible endpoints; runs in standard open harnesses (OpenHands, mini-SWE-agent)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Function calling, structured outputs; tuned for TauBench-style conversational tool use (V3 avg 70.9); MCP via harness</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M12" t="n">
+        <v>3316038765601</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Optimized for high-throughput agentic serving (300+ tok/s on Blackwell).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Qwen: Qwen3.7 Max</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Alibaba (Qwen)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Qwen Chat; DashScope / Model Studio API</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Native OpenAI + Anthropic API compatibility (works in Claude Code / Codex-style harnesses)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Function calling, extended thinking with preserve_thinking across turns, prompt caching; MCP (leads MCP-Mark per Alibaba); 35h autonomous kernel-optimization run (1,158 tool calls) reported</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M13" t="n">
+        <v>162911604779</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Agent-first positioning; API-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Xiaomi: MiMo-V2.5</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Xiaomi</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Xiaomi AI Studio; MiMo API (Token Plans)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible; SGLang/vLLM ship a dedicated 'mimo' tool-call parser for self-hosting</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Function calling; omnimodal input (text+image+audio+video) usable inside tool loops; MCP</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>audio+image+text+video</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>1048576</v>
+      </c>
+      <c r="M14" t="n">
+        <v>8676656451532</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Highest-volume open model on OpenRouter after Hy3; ~110M tool calls/week.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tencent: Hy3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tencent</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Tencent Yuanbao apps; Tencent Cloud API</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible; hosted by GMICloud, Novita, DeepInfra, SiliconFlow etc.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Function calling, structured outputs; MCP via harness</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>262144</v>
+      </c>
+      <c r="M15" t="n">
+        <v>9789999099848</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Free promo tier drove ~140M tool calls/week at peak; 295B/21B MoE (192 experts, top-8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Google: Gemini 3 Flash Preview</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Gemini CLI; AI Studio; Vertex AI Agent Builder</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Vertex/AI Studio APIs; Gemini CLI is open-source</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Google Search grounding, code execution, URL context, function calling; MCP</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>audio+file+image+text+video</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>1048576</v>
+      </c>
+      <c r="M16" t="n">
+        <v>947095724274</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Google's high-volume agentic workhorse tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Google: Gemini 3.1 Pro Preview</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Gemini CLI; AI Studio; Vertex AI</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Same Google API surfaces</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Google Search grounding, code execution, computer use (preview), function calling; MCP</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>audio+file+image+text+video</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>1048576</v>
+      </c>
+      <c r="M17" t="n">
+        <v>187952969447</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Tops hard-reasoning benchmarks (GPQA 94.3) but trails on agentic harness benchmarks (Terminal-Bench 74.0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>xAI: Grok 4.5</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Grok Build (xAI's coding-agent harness); Grok apps / X integration</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible xAI API</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Real-time X/web search, code execution, function calling; MCP</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>file+image+text</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>500000</v>
+      </c>
+      <c r="M18" t="n">
+        <v>336085799788</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>AA benchmarks it as the Grok 4.5 + Grok Build pair (ties Sol on SWE-Atlas-QnA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Meta: Llama 4 Maverick</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>None (no first-party agent product); Meta AI consumer apps use tuned variants</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Served by 20+ clouds; used in open harnesses (OpenHands, custom agents)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Function calling and structured outputs only - no reasoning-effort controls exposed (pre-reasoning-era design)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>image+text</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>1048576</v>
+      </c>
+      <c r="M19" t="n">
+        <v>34890889531</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2025-generation model; still significant volume as a cheap workhorse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>OpenAI: gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>None first-party; reference Harmony chat format</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Runs in most open harnesses; served by 20 providers</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Function calling, structured outputs, reasoning effort controls; browser/python tool support in the Harmony format</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>131072</v>
+      </c>
+      <c r="M20" t="n">
+        <v>565669378056</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>OpenAI's open-weights line (Apache 2.0); no first-party agent product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>StepFun: Step 3.7 Flash</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>StepFun</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>open-weights</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>StepFun API / apps</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Function calling, structured outputs, reasoning; video input; MCP via harness</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>image+text+video</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>256000</v>
+      </c>
+      <c r="M21" t="n">
+        <v>893527077750</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Budget agentic tier; 894B tokens/week on OpenRouter.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N21"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -22051,7 +24141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22787,7 +24877,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23386,7 +25476,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23928,629 +26018,4 @@
   <autoFilter ref="A1:M11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>developer</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>class</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>total_params_b</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>pretraining_tokens_t</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>tokens_per_total_param</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>disclosure_status</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Kimi K3</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Moonshot AI</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Undisclosed (tech report due with weights, 2026-07-27)</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Pipeline disclosed without quantities: web+code+vision pretraining, long-context mid-training toward 1M, SFT, RLVR. Predecessor Kimi K2 (1T params) disclosed 15.5T tokens, so K3's corpus is presumably well beyond that; treat any specific figure circulating now as an estimate.</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>kimi.com/blog/kimi-k3; Kimi K2 paper (arXiv:2507.20534)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Kimi K2 / K2.6</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Moonshot AI</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E3" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="F3" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Disclosed for K2 base (K2.6/K2.7 increments not broken out)</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>15.5T curated tokens across web text, code, mathematics, knowledge; MuonClip optimizer, 4,096-token pretraining window.</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Kimi K2 paper (arXiv:2507.20534)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Claude Fable 5</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Anthropic</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>closed</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Anthropic discloses neither corpus size nor parameter count for any frontier model.</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Fable 5 system card (no training-data quantities)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>GPT-5.6 Sol</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>closed</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>OpenAI stopped disclosing training-data scale after GPT-3 (300B tokens, 2020). gpt-oss open-weight models also ship without a precise token count ('trillions of tokens').</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>GPT-5.6 launch materials (no training-data quantities)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Gemini 3.x</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>closed</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>No corpus quantities disclosed for the Gemini series.</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Gemini model cards</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>GLM-5 / 5.1 / 5.2</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Z.ai (Zhipu)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>753</v>
-      </c>
-      <c r="E7" t="n">
-        <v>27</v>
-      </c>
-      <c r="F7" t="n">
-        <v>35.9</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Disclosed (GLM-5 base, which 5.1/5.2 build on)</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>27T-token corpus prioritizing code and reasoning early; distinct mid-training phase extends context 4K-&gt;200K with long-context agentic data.</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>GLM-5 paper (arXiv:2602.15763)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>DeepSeek V4 Pro</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>DeepSeek</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1600</v>
-      </c>
-      <c r="E8" t="n">
-        <v>32</v>
-      </c>
-      <c r="F8" t="n">
-        <v>20</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Disclosed ('more than 32T tokens', shared corpus with Flash)</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Agentic tool-use data injected already in mid-training; FP8-mixed pretraining with MXFP4 on expert weights.</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>DeepSeek-V4 report (arXiv:2606.19348)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>DeepSeek V4 Flash</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DeepSeek</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>284</v>
-      </c>
-      <c r="E9" t="n">
-        <v>32</v>
-      </c>
-      <c r="F9" t="n">
-        <v>112.7</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Disclosed ('more than 32T tokens', shared corpus with Pro)</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Same &gt;32T corpus as V4 Pro; the small variant is heavily over-trained relative to its size (~113 tokens per param).</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>DeepSeek-V4 report (arXiv:2606.19348)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Qwen3.7 Max</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Alibaba (Qwen)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>closed</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Undisclosed (closed tier)</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Alibaba disclosed 36T tokens for the open Qwen3 generation (2025) but publishes no quantities for the closed Max tier.</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Qwen3 technical report (2025); Qwen3.7 launch blog</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Nemotron 3 (Nano/Super/Ultra)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>NVIDIA</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>25</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Disclosed AND largely released - the only lab that ships much of the corpus itself</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>25T tokens in two phases (23.5T diverse + 1.5T high-quality) + 121B long-context phase; 16 data categories. ~8-10T tokens (~40-50% of the blend) released as open datasets (Nemotron-CC-v2.x, CC-Math, Pretraining-Code, Specialized). Documented for Nano/Super; Ultra follows the same data program.</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>NVIDIA Nemotron 3 pretraining docs + Nano tech report; HF Nemotron pretraining dataset collections</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>MiMo-V2.5</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Xiaomi</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>310</v>
-      </c>
-      <c r="E12" t="n">
-        <v>48</v>
-      </c>
-      <c r="F12" t="n">
-        <v>154.8</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Disclosed - largest disclosed corpus of any model here</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>~48T tokens, FP8 mixed precision, five-stage pipeline (text pretraining, projector warmup, multimodal pretraining, SFT/agentic post-training with 32K-&gt;256K-&gt;1M context extension, RL+MOPD). ~155 tokens per param - the most over-trained large model on this list.</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>XiaomiMiMo/MiMo-V2.5 HF card; mimo.xiaomi.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Hy3</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Tencent</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>295</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>295B/21B MoE (192 experts, top-8 routing); Tencent's model card discusses post-training scale-up but no corpus count.</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Tencent Hy3 model card; SiliconFlow explainer</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>MiniMax M3</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>MiniMax</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>No corpus size published for M3; total params also not officially stated (third-party estimates ~200-400B).</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>M3 launch materials</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Llama 4 Scout</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>109</v>
-      </c>
-      <c r="E15" t="n">
-        <v>40</v>
-      </c>
-      <c r="F15" t="n">
-        <v>367</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Disclosed (2025)</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>~40T multimodal tokens - highest tokens-per-param ratio here (~367x); 10M-token context via iRoPE.</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Meta Llama 4 launch blog (2025)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Llama 4 Maverick</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>open-weights</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>400</v>
-      </c>
-      <c r="E16" t="n">
-        <v>22</v>
-      </c>
-      <c r="F16" t="n">
-        <v>55</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Disclosed (2025)</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>~22T multimodal tokens.</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Meta Llama 4 launch blog (2025)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I16"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>